<commit_message>
Add Math sample exam with bold red answers for DOCX and PDF, and update UI sample download options
</commit_message>
<xml_diff>
--- a/exports/Bang_dap_an_tong_hop.xlsx
+++ b/exports/Bang_dap_an_tong_hop.xlsx
@@ -53,13 +53,13 @@
     <font>
       <name val="Times New Roman"/>
       <b val="1"/>
-      <color rgb="004B5563"/>
+      <color rgb="00047857"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Times New Roman"/>
       <b val="1"/>
-      <color rgb="00047857"/>
+      <color rgb="004B5563"/>
       <sz val="11"/>
     </font>
     <font>
@@ -607,22 +607,22 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -634,22 +634,22 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -661,22 +661,22 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -688,22 +688,22 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -715,17 +715,17 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -747,17 +747,17 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -828,22 +828,22 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Đ</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Đ</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Đ</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Đ</t>
+          <t>S</t>
         </is>
       </c>
     </row>
@@ -855,22 +855,22 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Đ</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>Đ</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>Đ</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Đ</t>
         </is>
       </c>
     </row>
@@ -882,22 +882,22 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Đ</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Đ</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Đ</t>
         </is>
       </c>
     </row>
@@ -909,22 +909,22 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Đ</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="inlineStr">
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Đ</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>Đ</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>Đ</t>
+          <t>S</t>
         </is>
       </c>
     </row>
@@ -936,20 +936,20 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Đ</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>Đ</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -963,20 +963,20 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Đ</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="D9" s="11" t="inlineStr">
-        <is>
-          <t>Đ</t>
-        </is>
-      </c>
-      <c r="E9" s="11" t="inlineStr">
+          <t>Đ</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Đ</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>Đ</t>
         </is>
@@ -990,20 +990,20 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>Đ</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
+          <t>Đ</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Đ</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -1017,20 +1017,20 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Đ</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Đ</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="E11" s="11" t="inlineStr">
+          <t>Đ</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>Đ</t>
         </is>
@@ -1103,22 +1103,22 @@
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
           <t>12</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>3</t>
         </is>
       </c>
     </row>
@@ -1130,22 +1130,22 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
           <t>3</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>9</t>
         </is>
       </c>
     </row>
@@ -1162,17 +1162,17 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Support variation tables, function graphs, and science diagrams across PDF/DOCX parsing, shuffling, and export
</commit_message>
<xml_diff>
--- a/exports/Bang_dap_an_tong_hop.xlsx
+++ b/exports/Bang_dap_an_tong_hop.xlsx
@@ -53,13 +53,13 @@
     <font>
       <name val="Times New Roman"/>
       <b val="1"/>
-      <color rgb="00047857"/>
+      <color rgb="004B5563"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Times New Roman"/>
       <b val="1"/>
-      <color rgb="004B5563"/>
+      <color rgb="00047857"/>
       <sz val="11"/>
     </font>
     <font>
@@ -174,10 +174,10 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -612,7 +612,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -644,12 +644,12 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -661,22 +661,22 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -688,22 +688,22 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
           <t>B</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
         </is>
       </c>
     </row>
@@ -715,14 +715,14 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
           <t>B</t>
@@ -730,7 +730,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -742,22 +742,22 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>A</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>B</t>
         </is>
       </c>
     </row>
@@ -828,22 +828,22 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Đ</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Đ</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Đ</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Đ</t>
         </is>
       </c>
     </row>
@@ -858,14 +858,14 @@
           <t>Đ</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="D5" s="11" t="inlineStr">
-        <is>
-          <t>S</t>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Đ</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Đ</t>
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
@@ -882,22 +882,22 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
+          <t>Đ</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Đ</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Đ</t>
+          <t>S</t>
         </is>
       </c>
     </row>
@@ -934,24 +934,24 @@
           <t>Câu 2.a</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
+          <t>Đ</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Đ</t>
         </is>
       </c>
     </row>
@@ -966,9 +966,9 @@
           <t>Đ</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>Đ</t>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
@@ -976,9 +976,9 @@
           <t>Đ</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
-        <is>
-          <t>Đ</t>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
         </is>
       </c>
     </row>
@@ -988,22 +988,22 @@
           <t>Câu 2.c</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Đ</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>Đ</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Đ</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Đ</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -1108,17 +1108,17 @@
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
           <t>9</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>9</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>12</t>
         </is>
       </c>
     </row>
@@ -1167,12 +1167,12 @@
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
     </row>

</xml_diff>